<commit_message>
Update Solar91 ONM portal and tests
</commit_message>
<xml_diff>
--- a/frontend/static/templates/PM_Task_Plan_Template.xlsx
+++ b/frontend/static/templates/PM_Task_Plan_Template.xlsx
@@ -531,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:C24"/>
+  <dimension ref="B2:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="3" customWidth="1" style="27" min="1" max="1"/>
@@ -634,7 +634,7 @@
       </c>
       <c r="C11" s="29" t="inlineStr">
         <is>
-          <t>First date the task is due. Type as DD-MM-YYYY or YYYY-MM-DD. Next dates are calculated from Frequency.</t>
+          <t>First date the task is due. Type as DD-MM-YYYY or YYYY-MM-DD. Next dates are calculated from Frequency. When the upload is set to follow the 30-day PM cycle, this is the cycle start (day 1) and the portal sets each equipment's dates from its turn: Plant side Inverter days 1-7, ACCB Panel + MCCB 8-9, VCB Panel 10-11, Transformer (IDT) 12-13, Aux. Transformer 14-15, 4 Pole 16-17, Earthing 18-19, other equipment 20-22, Transmission line 23-24; GSS side VCB 25-26, 4 Pole 27-28, Transmission line 29-30. Leave blank to use the cycle start chosen in the portal.</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19" ht="30" customHeight="1" s="27">
       <c r="B19" s="10" t="inlineStr">
         <is>
@@ -6369,7 +6368,7 @@
   </sheetData>
   <dataValidations count="5">
     <dataValidation sqref="A2:A301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>=Lists!$A$2:$A$24</formula1>
+      <formula1>=Lists!$A$2:$A$26</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D301" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Lists!$B$2:$B$7</formula1>
@@ -7884,50 +7883,58 @@
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
         <is>
-          <t>Boundary wall</t>
+          <t>4 Pole - GSS side</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
         <is>
-          <t>Water pipe line</t>
+          <t>Transmission line - GSS side</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="27">
       <c r="A21" s="23" t="inlineStr">
         <is>
-          <t>Vegetation</t>
+          <t>Boundary wall</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="27">
       <c r="A22" s="23" t="inlineStr">
         <is>
-          <t>Street Light</t>
+          <t>Water pipe line</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="27">
       <c r="A23" s="23" t="inlineStr">
         <is>
-          <t>BIKE</t>
+          <t>Vegetation</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="27">
       <c r="A24" s="23" t="inlineStr">
         <is>
+          <t>Street Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1" s="27">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>BIKE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1" s="27">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
           <t>Other</t>
         </is>
       </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="27">
-      <c r="A25" s="23" t="n"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="27">
-      <c r="A26" s="23" t="n"/>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="27">
       <c r="A27" s="23" t="n"/>

</xml_diff>